<commit_message>
feat(scripts): basic NGAF extraction script + value updates
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/14-electricity.xlsx
+++ b/packages/calculators/src/modules/test/14-electricity.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators-internal/packages/calculators/src/modules/test/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20066D07-B7A9-FD4E-8E1A-6773CAF67D66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27BA3B66-F57E-3448-BA5C-F3FCD1B335D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15900" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
@@ -957,19 +957,19 @@
       <c r="D5" s="11"/>
       <c r="E5" s="11">
         <f t="shared" ref="E5:E13" si="0">IF(ISBLANK(A5), "", VLOOKUP(B5, $P$20:$T$28, 2, FALSE))</f>
-        <v>0.66</v>
+        <v>0.6</v>
       </c>
       <c r="F5" s="11">
         <f>IF(ISBLANK(A5), "", VLOOKUP(B5, $P$20:$T$28, 4, FALSE))</f>
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G5" s="11">
         <f>$Q$15</f>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H5" s="11">
         <f>$R$15</f>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I5" s="11">
         <f t="shared" ref="I5:I13" si="1">IF(ISBLANK(A5), "", IF(B5="act", $Q$5, 0))</f>
@@ -981,12 +981,12 @@
       </c>
       <c r="K5" s="11">
         <f>A5*E5/1000</f>
-        <v>0.66</v>
+        <v>0.6</v>
       </c>
       <c r="L5" s="11"/>
       <c r="M5" s="11">
         <f>IF(ISBLANK(A5), "", A5*F5/1000)</f>
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="N5" s="11"/>
       <c r="O5" s="11"/>
@@ -1010,19 +1010,19 @@
       <c r="D6" s="11"/>
       <c r="E6" s="11">
         <f t="shared" si="0"/>
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="F6" s="11">
         <f t="shared" ref="F6:F23" si="2">IF(ISBLANK(A6), "", VLOOKUP(B6, $P$20:$T$28, 4, FALSE))</f>
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="G6" s="11">
         <f t="shared" ref="G6:G13" si="3">$Q$15</f>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H6" s="11">
         <f t="shared" ref="H6:H23" si="4">$R$15</f>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I6" s="11">
         <f t="shared" si="1"/>
@@ -1034,12 +1034,12 @@
       </c>
       <c r="K6" s="11">
         <f t="shared" ref="K6:K13" si="6">A6*E6/1000</f>
-        <v>1.54</v>
+        <v>1.48</v>
       </c>
       <c r="L6" s="11"/>
       <c r="M6" s="11">
         <f t="shared" ref="M6:M14" si="7">IF(ISBLANK(A6), "", A6*F6/1000)</f>
-        <v>0.18</v>
+        <v>0.22</v>
       </c>
       <c r="N6" s="11"/>
       <c r="O6" s="11"/>
@@ -1054,19 +1054,19 @@
       <c r="D7" s="11"/>
       <c r="E7" s="11">
         <f t="shared" si="0"/>
-        <v>0.71</v>
+        <v>0.65</v>
       </c>
       <c r="F7" s="11">
         <f t="shared" si="2"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="G7" s="11">
         <f t="shared" si="3"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H7" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I7" s="11">
         <f t="shared" si="1"/>
@@ -1078,12 +1078,12 @@
       </c>
       <c r="K7" s="11">
         <f t="shared" si="6"/>
-        <v>2.13</v>
+        <v>1.95</v>
       </c>
       <c r="L7" s="11"/>
       <c r="M7" s="11">
         <f t="shared" si="7"/>
-        <v>0.3</v>
+        <v>0.33</v>
       </c>
       <c r="N7" s="11"/>
       <c r="O7" s="11"/>
@@ -1098,19 +1098,19 @@
       <c r="D8" s="11"/>
       <c r="E8" s="11">
         <f t="shared" si="0"/>
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="F8" s="11">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="G8" s="11">
         <f t="shared" si="3"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H8" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I8" s="11">
         <f t="shared" si="1"/>
@@ -1122,12 +1122,12 @@
       </c>
       <c r="K8" s="11">
         <f t="shared" si="6"/>
-        <v>0.92</v>
+        <v>0.84</v>
       </c>
       <c r="L8" s="11"/>
       <c r="M8" s="11">
         <f t="shared" si="7"/>
-        <v>0.2</v>
+        <v>0.12</v>
       </c>
       <c r="N8" s="11"/>
       <c r="O8" s="11"/>
@@ -1142,19 +1142,19 @@
       <c r="D9" s="11"/>
       <c r="E9" s="11">
         <f t="shared" si="0"/>
-        <v>0.51</v>
+        <v>0.45</v>
       </c>
       <c r="F9" s="11">
         <f t="shared" si="2"/>
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="G9" s="11">
         <f t="shared" si="3"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H9" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I9" s="11">
         <f t="shared" si="1"/>
@@ -1166,12 +1166,12 @@
       </c>
       <c r="K9" s="11">
         <f t="shared" si="6"/>
-        <v>2.5499999999999998</v>
+        <v>2.25</v>
       </c>
       <c r="L9" s="11"/>
       <c r="M9" s="11">
         <f t="shared" si="7"/>
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="N9" s="11"/>
     </row>
@@ -1185,7 +1185,7 @@
       <c r="D10" s="11"/>
       <c r="E10" s="11">
         <f t="shared" si="0"/>
-        <v>0.61</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="F10" s="11">
         <f t="shared" si="2"/>
@@ -1193,11 +1193,11 @@
       </c>
       <c r="G10" s="11">
         <f t="shared" si="3"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H10" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I10" s="11">
         <f t="shared" si="1"/>
@@ -1209,7 +1209,7 @@
       </c>
       <c r="K10" s="11">
         <f t="shared" si="6"/>
-        <v>3.66</v>
+        <v>3.3600000000000003</v>
       </c>
       <c r="L10" s="11"/>
       <c r="M10" s="11">
@@ -1228,7 +1228,7 @@
       <c r="D11" s="11"/>
       <c r="E11" s="11">
         <f t="shared" si="0"/>
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="F11" s="11">
         <f t="shared" si="2"/>
@@ -1236,11 +1236,11 @@
       </c>
       <c r="G11" s="11">
         <f t="shared" si="3"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H11" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I11" s="11">
         <f t="shared" si="1"/>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="K11" s="11">
         <f t="shared" si="6"/>
-        <v>1.05</v>
+        <v>1.47</v>
       </c>
       <c r="L11" s="11"/>
       <c r="M11" s="11">
@@ -1271,19 +1271,19 @@
       <c r="D12" s="11"/>
       <c r="E12" s="11">
         <f t="shared" si="0"/>
-        <v>0.56000000000000005</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="F12" s="11">
         <f t="shared" si="2"/>
-        <v>7.0000000000000007E-2</v>
+        <v>0.13</v>
       </c>
       <c r="G12" s="11">
         <f t="shared" si="3"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H12" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I12" s="11">
         <f t="shared" si="1"/>
@@ -1295,12 +1295,12 @@
       </c>
       <c r="K12" s="11">
         <f t="shared" si="6"/>
-        <v>4.4800000000000004</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="L12" s="11"/>
       <c r="M12" s="11">
         <f t="shared" si="7"/>
-        <v>0.56000000000000005</v>
+        <v>1.04</v>
       </c>
       <c r="N12" s="11"/>
     </row>
@@ -1315,19 +1315,19 @@
       <c r="D13" s="11"/>
       <c r="E13" s="11">
         <f t="shared" si="0"/>
-        <v>0.66</v>
+        <v>0.6</v>
       </c>
       <c r="F13" s="11">
         <f t="shared" si="2"/>
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G13" s="11">
         <f t="shared" si="3"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H13" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I13" s="11">
         <f t="shared" si="1"/>
@@ -1339,12 +1339,12 @@
       </c>
       <c r="K13" s="11">
         <f t="shared" si="6"/>
-        <v>5.94</v>
+        <v>5.4</v>
       </c>
       <c r="L13" s="11"/>
       <c r="M13" s="11">
         <f t="shared" si="7"/>
-        <v>0.36</v>
+        <v>0.63000000000000012</v>
       </c>
       <c r="N13" s="11"/>
       <c r="O13" s="11"/>
@@ -1404,19 +1404,19 @@
       </c>
       <c r="E15" s="11">
         <f t="shared" ref="E15:E23" si="10">IF(ISBLANK(A15), "", VLOOKUP(B15, $P$20:$T$28, 2, FALSE))</f>
-        <v>0.66</v>
+        <v>0.6</v>
       </c>
       <c r="F15" s="11">
         <f t="shared" si="2"/>
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G15" s="11">
         <f>$Q$15</f>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H15" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I15" s="11">
         <f t="shared" ref="I15:I23" si="11">IF(ISBLANK(A15), "", IF(B15="act", $Q$5, 0))</f>
@@ -1429,22 +1429,22 @@
       <c r="K15" s="11"/>
       <c r="L15" s="11">
         <f>IF(ISBLANK(A15), "", J15*G15/1000)</f>
-        <v>0.43197300000000005</v>
+        <v>0.4213070000000001</v>
       </c>
       <c r="M15" s="11"/>
       <c r="N15" s="11">
         <f t="shared" si="9"/>
-        <v>5.3330000000000009E-2</v>
+        <v>5.8663000000000014E-2</v>
       </c>
       <c r="O15" s="11"/>
       <c r="P15" t="s">
         <v>9</v>
       </c>
       <c r="Q15">
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="R15">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -1462,19 +1462,19 @@
       </c>
       <c r="E16" s="11">
         <f t="shared" si="10"/>
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="F16" s="11">
         <f t="shared" si="2"/>
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
       <c r="G16" s="11">
         <f t="shared" ref="G16:G23" si="12">$Q$15</f>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H16" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I16" s="11">
         <f t="shared" si="11"/>
@@ -1487,12 +1487,12 @@
       <c r="K16" s="11"/>
       <c r="L16" s="11">
         <f t="shared" si="8"/>
-        <v>2.5378920000000003</v>
+        <v>2.4752280000000004</v>
       </c>
       <c r="M16" s="11"/>
       <c r="N16" s="11">
         <f t="shared" si="9"/>
-        <v>0.31332000000000004</v>
+        <v>0.34465200000000007</v>
       </c>
       <c r="O16" s="11"/>
     </row>
@@ -1511,19 +1511,19 @@
       </c>
       <c r="E17" s="11">
         <f t="shared" si="10"/>
-        <v>0.71</v>
+        <v>0.65</v>
       </c>
       <c r="F17" s="11">
         <f t="shared" si="2"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="G17" s="11">
         <f t="shared" si="12"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H17" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I17" s="11">
         <f t="shared" si="11"/>
@@ -1536,12 +1536,12 @@
       <c r="K17" s="11"/>
       <c r="L17" s="11">
         <f t="shared" si="8"/>
-        <v>1.862919</v>
+        <v>1.816921</v>
       </c>
       <c r="M17" s="11"/>
       <c r="N17" s="11">
         <f t="shared" si="9"/>
-        <v>0.22999</v>
+        <v>0.25298900000000002</v>
       </c>
       <c r="O17" s="11"/>
     </row>
@@ -1560,19 +1560,19 @@
       </c>
       <c r="E18" s="11">
         <f t="shared" si="10"/>
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="F18" s="11">
         <f t="shared" si="2"/>
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="G18" s="11">
         <f t="shared" si="12"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H18" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I18" s="11">
         <f t="shared" si="11"/>
@@ -1585,12 +1585,12 @@
       <c r="K18" s="11"/>
       <c r="L18" s="11">
         <f t="shared" si="8"/>
-        <v>3.3478920000000008</v>
+        <v>3.2652280000000005</v>
       </c>
       <c r="M18" s="11"/>
       <c r="N18" s="11">
         <f t="shared" si="9"/>
-        <v>0.41332000000000013</v>
+        <v>0.45465200000000011</v>
       </c>
       <c r="O18" s="11"/>
     </row>
@@ -1609,19 +1609,19 @@
       </c>
       <c r="E19" s="11">
         <f t="shared" si="10"/>
-        <v>0.51</v>
+        <v>0.45</v>
       </c>
       <c r="F19" s="11">
         <f t="shared" si="2"/>
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="G19" s="11">
         <f t="shared" si="12"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H19" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I19" s="11">
         <f t="shared" si="11"/>
@@ -1634,12 +1634,12 @@
       <c r="K19" s="11"/>
       <c r="L19" s="11">
         <f t="shared" si="8"/>
-        <v>2.5648650000000002</v>
+        <v>2.5015350000000005</v>
       </c>
       <c r="M19" s="11"/>
       <c r="N19" s="11">
         <f t="shared" si="9"/>
-        <v>0.31665000000000004</v>
+        <v>0.34831499999999999</v>
       </c>
       <c r="O19" s="11"/>
       <c r="P19" s="17" t="s">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="E20" s="11">
         <f t="shared" si="10"/>
-        <v>0.61</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="F20" s="11">
         <f t="shared" si="2"/>
@@ -1678,11 +1678,11 @@
       </c>
       <c r="G20" s="11">
         <f t="shared" si="12"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H20" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I20" s="11">
         <f t="shared" si="11"/>
@@ -1695,22 +1695,22 @@
       <c r="K20" s="11"/>
       <c r="L20" s="11">
         <f t="shared" si="8"/>
-        <v>3.1588380000000003</v>
+        <v>3.0808420000000001</v>
       </c>
       <c r="M20" s="11"/>
       <c r="N20" s="11">
         <f t="shared" si="9"/>
-        <v>0.38997999999999999</v>
+        <v>0.42897800000000003</v>
       </c>
       <c r="O20" s="11"/>
       <c r="P20" s="16" t="s">
         <v>33</v>
       </c>
       <c r="Q20">
-        <v>0.66</v>
+        <v>0.6</v>
       </c>
       <c r="S20">
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="21" spans="1:23">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="E21" s="11">
         <f t="shared" si="10"/>
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="F21" s="11">
         <f t="shared" si="2"/>
@@ -1736,11 +1736,11 @@
       </c>
       <c r="G21" s="11">
         <f t="shared" si="12"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H21" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I21" s="11">
         <f t="shared" si="11"/>
@@ -1753,22 +1753,22 @@
       <c r="K21" s="11"/>
       <c r="L21" s="11">
         <f t="shared" si="8"/>
-        <v>4.3198110000000005</v>
+        <v>4.2131490000000005</v>
       </c>
       <c r="M21" s="11"/>
       <c r="N21" s="11">
         <f t="shared" si="9"/>
-        <v>0.53331000000000006</v>
+        <v>0.58664100000000008</v>
       </c>
       <c r="O21" s="11"/>
       <c r="P21" s="16" t="s">
         <v>41</v>
       </c>
       <c r="Q21">
-        <v>0.66</v>
+        <v>0.6</v>
       </c>
       <c r="S21">
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="22" spans="1:23">
@@ -1786,19 +1786,19 @@
       </c>
       <c r="E22" s="11">
         <f t="shared" si="10"/>
-        <v>0.56000000000000005</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="F22" s="11">
         <f t="shared" si="2"/>
-        <v>7.0000000000000007E-2</v>
+        <v>0.13</v>
       </c>
       <c r="G22" s="11">
         <f t="shared" si="12"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H22" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I22" s="11">
         <f t="shared" si="11"/>
@@ -1811,21 +1811,21 @@
       <c r="K22" s="11"/>
       <c r="L22" s="11">
         <f t="shared" si="8"/>
-        <v>3.7797840000000007</v>
+        <v>3.6864560000000006</v>
       </c>
       <c r="M22" s="11"/>
       <c r="N22" s="11">
         <f t="shared" si="9"/>
-        <v>0.46664000000000011</v>
+        <v>0.51330400000000009</v>
       </c>
       <c r="P22" s="16" t="s">
         <v>34</v>
       </c>
       <c r="Q22">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="S22">
-        <v>0.09</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="23" spans="1:23">
@@ -1843,19 +1843,19 @@
       </c>
       <c r="E23" s="11">
         <f t="shared" si="10"/>
-        <v>0.66</v>
+        <v>0.6</v>
       </c>
       <c r="F23" s="11">
         <f t="shared" si="2"/>
-        <v>0.04</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="G23" s="11">
         <f t="shared" si="12"/>
-        <v>0.81</v>
+        <v>0.79</v>
       </c>
       <c r="H23" s="11">
         <f t="shared" si="4"/>
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="I23" s="11">
         <f t="shared" si="11"/>
@@ -1868,21 +1868,21 @@
       <c r="K23" s="11"/>
       <c r="L23" s="11">
         <f t="shared" si="8"/>
-        <v>3.54780000000001E-2</v>
+        <v>3.4602000000000105E-2</v>
       </c>
       <c r="M23" s="11"/>
       <c r="N23" s="11">
         <f t="shared" si="9"/>
-        <v>4.3800000000000124E-3</v>
+        <v>4.8180000000000141E-3</v>
       </c>
       <c r="P23" s="16" t="s">
         <v>35</v>
       </c>
       <c r="Q23">
-        <v>0.71</v>
+        <v>0.65</v>
       </c>
       <c r="S23">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="24" spans="1:23">
@@ -1890,10 +1890,10 @@
         <v>36</v>
       </c>
       <c r="Q24">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="S24">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="25" spans="1:23">
@@ -1902,10 +1902,10 @@
         <v>37</v>
       </c>
       <c r="Q25">
-        <v>0.51</v>
+        <v>0.45</v>
       </c>
       <c r="S25">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="26" spans="1:23">
@@ -1914,7 +1914,7 @@
         <v>38</v>
       </c>
       <c r="Q26">
-        <v>0.61</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="S26">
         <v>0.09</v>
@@ -1926,7 +1926,7 @@
         <v>39</v>
       </c>
       <c r="Q27">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="S27">
         <v>0.03</v>
@@ -1938,10 +1938,10 @@
         <v>40</v>
       </c>
       <c r="Q28">
-        <v>0.56000000000000005</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="S28">
-        <v>7.0000000000000007E-2</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="29" spans="1:23">
@@ -1950,10 +1950,10 @@
         <v>9</v>
       </c>
       <c r="Q29">
-        <v>0.63</v>
+        <v>0.59</v>
       </c>
       <c r="S29">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="30" spans="1:23">

</xml_diff>

<commit_message>
fix(constants): updated references and JRPP value
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/14-electricity.xlsx
+++ b/packages/calculators/src/modules/test/14-electricity.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27BA3B66-F57E-3448-BA5C-F3FCD1B335D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885DCABE-316C-2047-A8D7-4EC01BCF66F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="15900" xr2:uid="{5678E890-3691-CF46-80E7-00FB1F103661}"/>
   </bookViews>
@@ -989,7 +989,7 @@
         <v>14</v>
       </c>
       <c r="Q5">
-        <v>0.79510000000000003</v>
+        <v>0.76129999999999998</v>
       </c>
       <c r="R5" t="s">
         <v>20</v>
@@ -1326,11 +1326,11 @@
       </c>
       <c r="I13" s="11">
         <f t="shared" si="1"/>
-        <v>0.79510000000000003</v>
+        <v>0.76129999999999998</v>
       </c>
       <c r="J13" s="11">
         <f t="shared" si="5"/>
-        <v>343.80000000000013</v>
+        <v>648.00000000000057</v>
       </c>
       <c r="K13" s="11">
         <f t="shared" si="6"/>
@@ -1854,21 +1854,21 @@
       </c>
       <c r="I23" s="11">
         <f t="shared" si="11"/>
-        <v>0.79510000000000003</v>
+        <v>0.76129999999999998</v>
       </c>
       <c r="J23" s="11">
         <f t="shared" si="5"/>
-        <v>43.800000000000125</v>
+        <v>348.00000000000057</v>
       </c>
       <c r="K23" s="11"/>
       <c r="L23" s="11">
         <f t="shared" si="8"/>
-        <v>3.4602000000000105E-2</v>
+        <v>0.2749200000000005</v>
       </c>
       <c r="M23" s="11"/>
       <c r="N23" s="11">
         <f t="shared" si="9"/>
-        <v>4.8180000000000141E-3</v>
+        <v>3.8280000000000064E-2</v>
       </c>
       <c r="P23" s="16" t="s">
         <v>35</v>

</xml_diff>